<commit_message>
Rebuild one-pager — add ownership column and due dates
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -67,14 +67,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCEEFF"/>
-        <bgColor rgb="00DCEEFF"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -112,10 +112,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -489,36 +495,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Workstream</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>What Damco Handles</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>What Damco Does</t>
+          <t>What We Need From You</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>What We Need From Will</t>
+          <t>Due Date</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -526,393 +531,305 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Frequency</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="35" customHeight="1">
+    </row>
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>On-Page SEO</t>
+          <t>Blog — July post 1
+"Why Professional School Photography Matters"</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Blog Writing</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Damco writes the blog post and shares for review</t>
+          <t>Written and ready to publish</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Senthil to upload to website</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Review and approve the draft before publishing</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+          <t>ASAP</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Waiting on Senthil</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Blog — July post 2
+"Why School Photography Matters / What to Look for in a New Photographer"</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Writing in progress</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Review draft when shared, then approve</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>22 July 2026</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>2 per month</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="35" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>On-Page SEO</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Blog Publishing</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Will's team (Senthil) uploads approved blog to website</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Senthil to upload once Will approves</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Blog — "How to Choose a School Photography Company in the UK"</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Published on website — SEO audit done, fixes sent to Senthil</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Will to send corrected blog content</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Waiting on Will</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>FAQs</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Written and ready — schema code prepared for Senthil</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Will to complete review and approve</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Waiting on Will</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Website Fixes
+(Forms, CAPTCHA, Thank You pages)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Specifications sent to Senthil with full detail</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Senthil to implement and confirm live date</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Waiting on Senthil</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Quora</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Damco writes all answers — nothing for your team to write</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Review draft answers before we post — quick read and approve</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Ongoing — weekly</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>2 per month</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="35" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>On-Page SEO</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>FAQ Writing</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Damco writes FAQ answers and shares for review</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Review and approve answers before going live</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Done — pending publish</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>One-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="35" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>On-Page SEO</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>SEO Audit</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Damco audits published pages and sends fixes to Senthil</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>No action needed — Senthil handles fixes</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Reddit</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Damco writes all answers — nothing for your team to write</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Confirm the 3 questions shared are relevant topics for Imago</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>8 July 2026</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Waiting on Will</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Medium / Third-Party Articles</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Damco writes all articles and manages the account</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Review each article draft before we publish — approve or request changes</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SEO Audit — Blog Pages</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Damco audits all published blogs and sends fixes to Senthil</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>No action needed from Will's side</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="35" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>On-Page SEO</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Schema / Structured Data</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Damco prepares schema code and sends to Senthil</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>No action needed — Senthil adds the code</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Per page</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="35" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Technical SEO</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Website Fixes</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Damco identifies issues and shares with Senthil</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>No action needed — Senthil implements</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Monthly SEO Dashboard</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Damco prepares and shares every month</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Review the report — flag any questions</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>End of each month</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LLM Visibility
+(ChatGPT, Perplexity, Google AI)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Damco monitors and builds citations across platforms</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>No action needed from Will's side</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Monthly check — 31 July 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="35" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Off-Page SEO</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Quora</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Damco writes answers and shares drafts for approval</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Review and approve before posting</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="35" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Off-Page SEO</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Reddit</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Damco identifies questions and writes answers</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Review and confirm topics are relevant</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Pending Approval</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="35" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Off-Page SEO</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Third-Party Articles</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Damco writes articles and shares for approval</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Review and approve before anything goes live</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="35" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Off-Page SEO</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Business Directories</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Damco submits Imago to relevant directories</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>No action needed</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>One-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="35" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>AEO / GEO</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>LLM Visibility (ChatGPT / Perplexity)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Damco monitors and builds citations across platforms</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>No action needed</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Monthly check</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="35" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Reporting</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Monthly SEO Dashboard</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Damco prepares and shares monthly report</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Review the dashboard</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Monthly</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add dropdown menu to Status column in one-pager
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -834,6 +834,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid status" promptTitle="Status" prompt="Select a status" type="list">
+      <formula1>"In Progress,Waiting on Will,Waiting on Senthil,Done,Live,Planned"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 22 Jul 2026 call agenda sheet to one-pager
New tab with 8 agenda items — topic, discussion points, required outcome,
owner, and priority. Updates Reddit due date from overdue 8 July to 22 July.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="SEO Activity Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="22 Jul 2026 — Call Agenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +34,52 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00842029"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00664D03"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00155724"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +122,26 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -104,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,6 +194,33 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -715,7 +807,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>8 July 2026</t>
+          <t>22 July 2026</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -841,4 +933,295 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Call Agenda — Imago Photography  |  22 July 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Discussion Points</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>What We Need / Outcome</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="53" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>One-Pager Walkthrough</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>• Walk Will through each workstream — On-Page, Technical, Off-Page, AEO/GEO
+• Clarify what Damco handles vs what requires Will or Senthil
+• Confirm Will is comfortable with the approval process for Quora, Reddit, Medium</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Will confirms he has a clear picture of all activities and what his team needs to do</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Ashish</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Blog Update</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>• Blog 1 ("Why Professional School Photography Matters") — is it live yet? If not, get Senthil's timeline
+• Blog 2 ("Why School Photography Matters") — share writing update, confirm Will is reviewing</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Confirm live date for Blog 1. Get Will's approval on Blog 2 draft</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Ashish / Senthil</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="83" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Reddit Approval</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>• 3 questions shared — still pending Will's sign-off
+• r/photography — school photography discussion
+• r/Nikon — share Imago's images as brand expression
+• r/UKParenting — UK parents discussing school photo packages
+• Reminder: Damco writes everything, no time needed from Will's team</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Yes or no on each question — approval to post</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="53" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>SEO Audit Fixes</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>• Fixes sent to Senthil on 8 July — headings, internal links, meta title/description, alt text, schema
+• Without these fixes the blog will struggle to rank regardless of content quality
+• Confirm Senthil received the email and understands each fix</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Agree a deadline for all fixes to go live</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Senthil</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="68" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Medium / Third-Party Content</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>• Medium account live: medium.com/@MarketingSupport_61400
+• Confirm Will has the login details
+• Share first article draft for review if ready
+• Vocal.media is next platform after Medium — flag this</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Will confirms receipt of login. Approve or request changes on first draft</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Ashish / Will</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="53" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>August Blog Topics</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>• Recommend back-to-school angle — positions Imago for September search traffic
+• Suggest 2 topics for Will to approve today so writing can begin
+• Reminder: topics must be approved before writing starts</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Will approves 2 blog topics for August</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Ashish / Will</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="53" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Quora Update</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>• 2 answers posted this month — "How are large schools photographed?" and "How can parents prepare kids?"
+• Cadence: 1 per week, Damco shares draft before posting
+• Confirm Will is happy with the approval process</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Will confirms the process is working</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Ashish</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Actions Lock</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>• Agree all outstanding actions — owner and deadline for each
+• Key pending items: Blog 1 live date (Senthil), Reddit approval (Will), Blog 2 review (Will), SEO fixes deadline (Senthil)</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Every open action has a named owner and a date</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add GTM and web content agenda items to 22 Jul call sheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -941,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1218,6 +1218,65 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="53" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>GTM Implementation</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>• Google Tag Manager setup has been assigned to Senthil
+• Confirm Senthil has received the GTM requirements and access
+• Agree a go-live deadline for GTM to be implemented on the website</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Senthil confirms receipt and provides a live date for GTM implementation</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Senthil</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Web Page Content — Audit &amp; Pending Updates</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>• Damco shared content suggestions for multiple web pages
+• Following the audit, changes have been made on the School Photography page only
+• All remaining pages are still pending — content updates not yet applied
+• Agree which pages to prioritise next and set a timeline with Senthil</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Confirm remaining pages are on Senthil's list. Agree priority order and deadline for next batch of content updates</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Senthil / Ashish</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
Trim one-pager to single sheet — client-facing only
Removed Call Agenda and SEO Audit Priority Fixes tabs.
One-pager now contains only the SEO Activity Plan sheet.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -4,8 +4,6 @@
   <workbookPr/>
   <sheets>
     <sheet name="SEO Activity Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="22 Jul 2026 — Call Agenda" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SEO Audit — Priority Fixes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28909,567 +28907,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" style="28" min="1" max="1"/>
-    <col width="44" customWidth="1" style="28" min="2" max="2"/>
-    <col width="36" customWidth="1" style="28" min="3" max="3"/>
-    <col width="16" customWidth="1" style="28" min="4" max="4"/>
-    <col width="14" customWidth="1" style="28" min="5" max="5"/>
-    <col width="16" customWidth="1" style="28" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" s="28">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>Call Agenda — Imago Photography  |  22 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="28">
-      <c r="A2" s="30" t="inlineStr">
-        <is>
-          <t>Topic</t>
-        </is>
-      </c>
-      <c r="B2" s="30" t="inlineStr">
-        <is>
-          <t>Discussion Points</t>
-        </is>
-      </c>
-      <c r="C2" s="30" t="inlineStr">
-        <is>
-          <t>What We Need / Outcome</t>
-        </is>
-      </c>
-      <c r="D2" s="30" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="E2" s="30" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="F2" s="30" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="53" customHeight="1" s="28">
-      <c r="A3" s="31" t="inlineStr">
-        <is>
-          <t>Blog SEO — On-Page</t>
-        </is>
-      </c>
-      <c r="B3" s="32" t="inlineStr">
-        <is>
-          <t>• Blog 1 ("Why Professional School Photography Matters") — Will has shared both blogs for review
-• Blog 2 ("Why School Photography Matters") — review draft received
-• Confirm Senthil's live date for Blog 1 on website</t>
-        </is>
-      </c>
-      <c r="C3" s="33" t="inlineStr">
-        <is>
-          <t>Confirm live date for Blog 1. Get Will's approval on Blog 2 draft</t>
-        </is>
-      </c>
-      <c r="D3" s="34" t="inlineStr">
-        <is>
-          <t>Ashish</t>
-        </is>
-      </c>
-      <c r="E3" s="35" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F3" s="34" t="inlineStr">
-        <is>
-          <t>24 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="83" customHeight="1" s="28">
-      <c r="A4" s="31" t="inlineStr">
-        <is>
-          <t>Reddit Approval</t>
-        </is>
-      </c>
-      <c r="B4" s="32" t="inlineStr">
-        <is>
-          <t>• 3 questions shared — still pending Will's sign-off
-• r/photography — school photography discussion
-• r/Nikon — share Imago's images as brand expression
-• r/UKParenting — UK parents discussing school photo packages
-• Reminder: Damco writes everything, no time from Will's team needed</t>
-        </is>
-      </c>
-      <c r="C4" s="33" t="inlineStr">
-        <is>
-          <t>Yes or no on each question — approval to post</t>
-        </is>
-      </c>
-      <c r="D4" s="34" t="inlineStr">
-        <is>
-          <t>Will</t>
-        </is>
-      </c>
-      <c r="E4" s="35" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F4" s="34" t="inlineStr">
-        <is>
-          <t>29 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="53" customHeight="1" s="28">
-      <c r="A5" s="31" t="inlineStr">
-        <is>
-          <t>SEO Audit Fixes</t>
-        </is>
-      </c>
-      <c r="B5" s="32" t="inlineStr">
-        <is>
-          <t>• Fixes sent to Senthil on 8 July — headings, internal links, meta title/description, alt text, schema
-• Without these fixes the blog will not rank regardless of content quality
-• Fixes have been ranked by impact (see SEO Audit Priority sheet)</t>
-        </is>
-      </c>
-      <c r="C5" s="33" t="inlineStr">
-        <is>
-          <t>Agree a deadline for all fixes to go live</t>
-        </is>
-      </c>
-      <c r="D5" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-      <c r="E5" s="35" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>29 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="68" customHeight="1" s="28">
-      <c r="A6" s="31" t="inlineStr">
-        <is>
-          <t>Web Page Content — Pending Updates</t>
-        </is>
-      </c>
-      <c r="B6" s="32" t="inlineStr">
-        <is>
-          <t>• Damco shared content suggestions for multiple web pages
-• School Photography page — changes applied after audit
-• All remaining pages still pending — content updates not yet applied
-• Agree which pages to prioritise next</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Confirm remaining pages are on Senthil's list. Agree priority order and deadline for next batch</t>
-        </is>
-      </c>
-      <c r="D6" s="34" t="inlineStr">
-        <is>
-          <t>Senthil / Ashish</t>
-        </is>
-      </c>
-      <c r="E6" s="36" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>29 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="53" customHeight="1" s="28">
-      <c r="A7" s="31" t="inlineStr">
-        <is>
-          <t>August Blog Topics</t>
-        </is>
-      </c>
-      <c r="B7" s="32" t="inlineStr">
-        <is>
-          <t>• Recommend back-to-school angle — positions Imago for September search traffic
-• Suggest 2 topics for Will to approve today so writing can begin
-• Topics must be approved before writing starts</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
-          <t>Will approves 2 blog topics for August</t>
-        </is>
-      </c>
-      <c r="D7" s="34" t="inlineStr">
-        <is>
-          <t>Ashish / Will</t>
-        </is>
-      </c>
-      <c r="E7" s="36" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>29 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="53" customHeight="1" s="28">
-      <c r="A8" s="31" t="inlineStr">
-        <is>
-          <t>GTM Implementation</t>
-        </is>
-      </c>
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>• GTM setup assigned to Senthil
-• Thank You page part to be revised as part of this
-• Confirm Senthil has received requirements and access</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="inlineStr">
-        <is>
-          <t>Senthil confirms live date for GTM implementation</t>
-        </is>
-      </c>
-      <c r="D8" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-      <c r="E8" s="36" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>29 July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="53" customHeight="1" s="28">
-      <c r="A9" s="31" t="inlineStr">
-        <is>
-          <t>Quora Update</t>
-        </is>
-      </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>• 2 answers posted this month — "How are large schools photographed?" and "How can parents prepare kids?"
-• Cadence: 1 per week — Damco shares draft before posting
-• Will to share Quora drafts for review today</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>Will confirms approval process is working</t>
-        </is>
-      </c>
-      <c r="D9" s="34" t="inlineStr">
-        <is>
-          <t>Ashish</t>
-        </is>
-      </c>
-      <c r="E9" s="37" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" style="28" min="1" max="1"/>
-    <col width="44" customWidth="1" style="28" min="2" max="2"/>
-    <col width="20" customWidth="1" style="28" min="3" max="3"/>
-    <col width="20" customWidth="1" style="28" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" s="28">
-      <c r="A1" s="38" t="inlineStr">
-        <is>
-          <t>SEO Audit — Blog Fixes Ranked by Impact  |  How to Choose a School Photography Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="28">
-      <c r="A2" s="39" t="inlineStr">
-        <is>
-          <t>Fixes are ranked in order of SEO impact. Start with Critical — these have the highest effect on rankings. Do Important next. Good to have can wait.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" s="28">
-      <c r="A3" s="30" t="inlineStr">
-        <is>
-          <t>Fix Required</t>
-        </is>
-      </c>
-      <c r="B3" s="30" t="inlineStr">
-        <is>
-          <t>Why It Matters</t>
-        </is>
-      </c>
-      <c r="C3" s="30" t="inlineStr">
-        <is>
-          <t>Impact Level</t>
-        </is>
-      </c>
-      <c r="D3" s="30" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1" s="28">
-      <c r="A4" s="31" t="inlineStr">
-        <is>
-          <t>3 H1 tags on the page (should be 1 only)</t>
-        </is>
-      </c>
-      <c r="B4" s="32" t="inlineStr">
-        <is>
-          <t>Multiple H1s split ranking signals — search engines cannot determine the primary topic of the page</t>
-        </is>
-      </c>
-      <c r="C4" s="35" t="inlineStr">
-        <is>
-          <t>Critical — do first</t>
-        </is>
-      </c>
-      <c r="D4" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1" s="28">
-      <c r="A5" s="31" t="inlineStr">
-        <is>
-          <t>Article title coded as H3 instead of H2</t>
-        </is>
-      </c>
-      <c r="B5" s="32" t="inlineStr">
-        <is>
-          <t>Heading hierarchy must flow H1 → H2 → H3. Incorrect structure reduces how well search engines read the content</t>
-        </is>
-      </c>
-      <c r="C5" s="35" t="inlineStr">
-        <is>
-          <t>Critical — do first</t>
-        </is>
-      </c>
-      <c r="D5" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1" s="28">
-      <c r="A6" s="31" t="inlineStr">
-        <is>
-          <t>All section headings are H3 — no H2 used</t>
-        </is>
-      </c>
-      <c r="B6" s="32" t="inlineStr">
-        <is>
-          <t>Page jumps from H1 straight to H3 with no H2, breaking content structure for search engines</t>
-        </is>
-      </c>
-      <c r="C6" s="35" t="inlineStr">
-        <is>
-          <t>Critical — do first</t>
-        </is>
-      </c>
-      <c r="D6" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1" s="28">
-      <c r="A7" s="31" t="inlineStr">
-        <is>
-          <t>No Article schema on the page</t>
-        </is>
-      </c>
-      <c r="B7" s="32" t="inlineStr">
-        <is>
-          <t>Schema helps search engines understand the content type and can improve how the page appears in results</t>
-        </is>
-      </c>
-      <c r="C7" s="35" t="inlineStr">
-        <is>
-          <t>Critical — do first</t>
-        </is>
-      </c>
-      <c r="D7" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1" s="28">
-      <c r="A8" s="31" t="inlineStr">
-        <is>
-          <t>Only 1 internal link — 10 more identified</t>
-        </is>
-      </c>
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>Internal links help search engines discover other pages and pass authority across the site</t>
-        </is>
-      </c>
-      <c r="C8" s="36" t="inlineStr">
-        <is>
-          <t>Important — do next</t>
-        </is>
-      </c>
-      <c r="D8" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1" s="28">
-      <c r="A9" s="31" t="inlineStr">
-        <is>
-          <t>Title tag is 74 characters (max 60)</t>
-        </is>
-      </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>Titles over 60 characters are cut off in search results, reducing click-through rates</t>
-        </is>
-      </c>
-      <c r="C9" s="36" t="inlineStr">
-        <is>
-          <t>Important — do next</t>
-        </is>
-      </c>
-      <c r="D9" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1" s="28">
-      <c r="A10" s="31" t="inlineStr">
-        <is>
-          <t>Meta description is 122 characters (min 150–160)</t>
-        </is>
-      </c>
-      <c r="B10" s="32" t="inlineStr">
-        <is>
-          <t>Short descriptions reduce click-through rates — search engines may auto-generate a less relevant snippet</t>
-        </is>
-      </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>Important — do next</t>
-        </is>
-      </c>
-      <c r="D10" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1" s="28">
-      <c r="A11" s="31" t="inlineStr">
-        <is>
-          <t>2 images missing alt text</t>
-        </is>
-      </c>
-      <c r="B11" s="32" t="inlineStr">
-        <is>
-          <t>Alt text helps search engines understand images and is required for accessibility compliance</t>
-        </is>
-      </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>Good to have — when ready</t>
-        </is>
-      </c>
-      <c r="D11" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1" s="28">
-      <c r="A12" s="31" t="inlineStr">
-        <is>
-          <t>No outbound links to credible sources</t>
-        </is>
-      </c>
-      <c r="B12" s="32" t="inlineStr">
-        <is>
-          <t>Authoritative content is expected to reference credible sources, particularly on trust-sensitive topics like safeguarding</t>
-        </is>
-      </c>
-      <c r="C12" s="37" t="inlineStr">
-        <is>
-          <t>Good to have — when ready</t>
-        </is>
-      </c>
-      <c r="D12" s="34" t="inlineStr">
-        <is>
-          <t>Senthil</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update one-pager with 22 Jul client call outcomes
Blog 1 & 2 due dates set to 25 Jul. Will's blog content shared for review noted.
Website fixes updated to include GTM and Thank You page. How to Choose blog
fixes ownership moved to Senthil. All due dates filled. Single sheet only.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -254,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -366,6 +366,18 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -709,22 +721,22 @@
 "Why Professional School Photography Matters"</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="40" t="inlineStr">
         <is>
-          <t>Written and ready to publish</t>
+          <t>Written and ready to publish — Will has shared blog content for review</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="40" t="inlineStr">
         <is>
-          <t>Senthil to upload to website</t>
+          <t>Senthil to upload to website once reviewed</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="40" t="inlineStr">
         <is>
-          <t>ASAP — discussed 22 Jul</t>
+          <t>25 July 2026</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="41" t="inlineStr">
         <is>
           <t>Waiting on Senthil</t>
         </is>
@@ -758,24 +770,24 @@
 "Why School Photography Matters / What to Look for in a New Photographer"</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="42" t="inlineStr">
         <is>
-          <t>Writing in progress</t>
+          <t>Writing in progress — draft to be shared with Will for approval</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="42" t="inlineStr">
         <is>
-          <t>Review draft when shared, then approve</t>
+          <t>Review and approve draft when shared</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="42" t="inlineStr">
         <is>
-          <t>24 July 2026</t>
+          <t>25 July 2026</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="41" t="inlineStr">
         <is>
-          <t>Waiting on Will</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F3" s="13" t="n"/>
@@ -806,24 +818,24 @@
           <t>Blog — "How to Choose a School Photography Company in the UK"</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="40" t="inlineStr">
         <is>
-          <t>Published on website — SEO audit done, fixes sent to Senthil</t>
+          <t>Published on website — SEO audit done, fixes sent to Senthil on 8 July</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="40" t="inlineStr">
         <is>
-          <t>Will to send corrected blog content</t>
+          <t>No action needed from Will — Senthil to implement fixes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="40" t="inlineStr">
         <is>
-          <t>ASAP</t>
+          <t>29 July 2026</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="43" t="inlineStr">
         <is>
-          <t>Waiting on Will</t>
+          <t>Waiting on Senthil</t>
         </is>
       </c>
       <c r="F4" s="13" t="n"/>
@@ -854,22 +866,22 @@
           <t>FAQs</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>Written and ready — schema code prepared for Senthil</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>Will to complete review and approve</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>ASAP</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="43" t="inlineStr">
         <is>
           <t>Waiting on Will</t>
         </is>
@@ -903,22 +915,22 @@
 (Forms, CAPTCHA, Thank You pages)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>Specifications sent to Senthil with full detail</t>
+          <t>Specifications sent to Senthil — GTM and Thank You page part to be revised</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="40" t="inlineStr">
         <is>
           <t>Senthil to implement and confirm live date</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>ASAP</t>
+          <t>29 July 2026</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="41" t="inlineStr">
         <is>
           <t>Waiting on Senthil</t>
         </is>
@@ -951,22 +963,22 @@
           <t>Quora</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
-          <t>Damco writes all answers — nothing for your team to write</t>
+          <t>Damco writes all answers — drafts shared with Will before posting</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
-          <t>Review draft answers before we post — quick read and approve</t>
+          <t>Review and approve draft answers — quick read and approve</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Ongoing — weekly</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="41" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -999,22 +1011,22 @@
           <t>Reddit</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>Damco writes all answers — nothing for your team to write</t>
+          <t>Damco writes all answers — 3 questions shared with Will for topic approval</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
-          <t>Confirm the 3 questions shared are relevant topics for Imago</t>
+          <t>Confirm the 3 questions are relevant — yes or no on each</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>29 July 2026</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="43" t="inlineStr">
         <is>
           <t>Waiting on Will</t>
         </is>
@@ -1047,22 +1059,22 @@
           <t>Medium / Third-Party Articles</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="42" t="inlineStr">
         <is>
-          <t>Damco writes all articles and manages the account</t>
+          <t>Damco writes all articles — Medium account live, first draft being prepared</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>Review each article draft before we publish — approve or request changes</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="41" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -1095,22 +1107,22 @@
           <t>SEO Audit — Blog Pages</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>Damco audits all published blogs and sends fixes to Senthil</t>
+          <t>Audits done — fixes sent to Senthil. Fixes ranked by priority (Critical / Important / Good to have)</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>No action needed from Will's side</t>
+          <t>No action needed from Will — Senthil implements fixes</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="40" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="41" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -1143,22 +1155,22 @@
           <t>Monthly SEO Dashboard</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="42" t="inlineStr">
         <is>
-          <t>Damco prepares and shares every month</t>
+          <t>Damco prepares and shares monthly — due 20th of each month</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Review the report — flag any questions</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
-          <t>End of each month</t>
+          <t>20 August 2026</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="41" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -1192,22 +1204,22 @@
 (ChatGPT, Perplexity, Google AI)</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
-          <t>Damco monitors and builds citations across platforms</t>
+          <t>Damco monitors Imago visibility in ChatGPT, Perplexity, and Google AI Overviews</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="40" t="inlineStr">
         <is>
           <t>No action needed from Will's side</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="40" t="inlineStr">
         <is>
-          <t>Monthly check — 31 July 2026</t>
+          <t>31 July 2026</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="41" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>

</xml_diff>

<commit_message>
Update SEO activity one-pager with 22 July call outcomes
- Restore How to Choose blog row: Will to send corrected content, Waiting on Will
- Blog 1: reflect Will shared content for review, Senthil to upload
- Blog 2: due date set to 25 July
- Website Fixes: GTM added to activity name and description
- SEO Audit: fixes noted as ranked Critical / Important / Good to have
- Single sheet only, 12 activities

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -820,22 +820,22 @@
       </c>
       <c r="B4" s="40" t="inlineStr">
         <is>
-          <t>Published on website — SEO audit done, fixes sent to Senthil on 8 July</t>
+          <t>Published on website — SEO audit done; fixes sent to Senthil on 8 July</t>
         </is>
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
-          <t>No action needed from Will — Senthil to implement fixes</t>
+          <t>Will to send corrected blog content</t>
         </is>
       </c>
       <c r="D4" s="40" t="inlineStr">
         <is>
-          <t>29 July 2026</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="E4" s="43" t="inlineStr">
         <is>
-          <t>Waiting on Senthil</t>
+          <t>Waiting on Will</t>
         </is>
       </c>
       <c r="F4" s="13" t="n"/>
@@ -912,12 +912,12 @@
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Website Fixes
-(Forms, CAPTCHA, Thank You pages)</t>
+(Forms, CAPTCHA, Thank You pages, GTM)</t>
         </is>
       </c>
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>Specifications sent to Senthil — GTM and Thank You page part to be revised</t>
+          <t>Specifications sent to Senthil — GTM and Thank You page implementation included</t>
         </is>
       </c>
       <c r="C6" s="40" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>Audits done — fixes sent to Senthil. Fixes ranked by priority (Critical / Important / Good to have)</t>
+          <t>Audits done — fixes ranked by priority (Critical / Important / Good to have) and sent to Senthil</t>
         </is>
       </c>
       <c r="C10" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Reprioritise one-pager based on 22 July call transcript
Reorganise into three sections per Harshit's direction on the call:
- Active: items Damco can action now (blogs, Quora, Reddit, Medium, audit, dashboard, LLM)
- Waiting on Will: Blog 1, How to Choose blog, FAQs
- Parked: website fixes (Forms, CAPTCHA, GTM) — low period only, target last week of August

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -143,8 +143,18 @@
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -219,8 +229,43 @@
         <fgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002980B9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F39C12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0095A5A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F3F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A252F"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border/>
     <border>
       <left style="thin">
@@ -250,11 +295,43 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -377,6 +454,38 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -657,37 +766,37 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="97.56999999999999" customWidth="1" style="28" min="1" max="1"/>
-    <col width="76" customWidth="1" style="28" min="2" max="2"/>
-    <col width="94.86" customWidth="1" style="28" min="3" max="3"/>
-    <col width="38.86" customWidth="1" style="28" min="4" max="4"/>
-    <col width="27.14" customWidth="1" style="28" min="5" max="5"/>
+    <col width="35" customWidth="1" style="28" min="1" max="1"/>
+    <col width="40" customWidth="1" style="28" min="2" max="2"/>
+    <col width="35" customWidth="1" style="28" min="3" max="3"/>
+    <col width="22" customWidth="1" style="28" min="4" max="4"/>
+    <col width="20" customWidth="1" style="28" min="5" max="5"/>
     <col width="8.859999999999999" customWidth="1" style="28" min="6" max="6"/>
     <col width="8.710000000000001" customWidth="1" style="28" min="7" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="28">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="28">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="44" t="inlineStr">
         <is>
           <t>What Damco Handles</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="44" t="inlineStr">
         <is>
           <t>What We Need From You</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="44" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="44" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -715,32 +824,15 @@
       <c r="Z1" s="2" t="n"/>
     </row>
     <row r="2" ht="14.25" customHeight="1" s="28">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>Blog — July post 1
-"Why Professional School Photography Matters"</t>
+          <t>ACTIVE — Damco actioning now</t>
         </is>
       </c>
-      <c r="B2" s="40" t="inlineStr">
-        <is>
-          <t>Written and ready to publish — Will has shared blog content for review</t>
-        </is>
-      </c>
-      <c r="C2" s="40" t="inlineStr">
-        <is>
-          <t>Senthil to upload to website once reviewed</t>
-        </is>
-      </c>
-      <c r="D2" s="40" t="inlineStr">
-        <is>
-          <t>25 July 2026</t>
-        </is>
-      </c>
-      <c r="E2" s="41" t="inlineStr">
-        <is>
-          <t>Waiting on Senthil</t>
-        </is>
-      </c>
+      <c r="B2" s="46" t="n"/>
+      <c r="C2" s="46" t="n"/>
+      <c r="D2" s="46" t="n"/>
+      <c r="E2" s="47" t="n"/>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
       <c r="H2" s="13" t="n"/>
@@ -763,29 +855,29 @@
       <c r="Y2" s="13" t="n"/>
       <c r="Z2" s="13" t="n"/>
     </row>
-    <row r="3" ht="14.25" customHeight="1" s="28">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="50" customHeight="1" s="28">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Blog — July post 2
 "Why School Photography Matters / What to Look for in a New Photographer"</t>
         </is>
       </c>
-      <c r="B3" s="42" t="inlineStr">
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>Writing in progress — draft to be shared with Will for approval</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
+      <c r="C3" s="49" t="inlineStr">
         <is>
           <t>Review and approve draft when shared</t>
         </is>
       </c>
-      <c r="D3" s="42" t="inlineStr">
+      <c r="D3" s="49" t="inlineStr">
         <is>
           <t>25 July 2026</t>
         </is>
       </c>
-      <c r="E3" s="41" t="inlineStr">
+      <c r="E3" s="49" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -812,30 +904,30 @@
       <c r="Y3" s="13" t="n"/>
       <c r="Z3" s="13" t="n"/>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="28">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="50" customHeight="1" s="28">
+      <c r="A4" s="48" t="inlineStr">
         <is>
-          <t>Blog — "How to Choose a School Photography Company in the UK"</t>
+          <t>Quora</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
+      <c r="B4" s="49" t="inlineStr">
         <is>
-          <t>Published on website — SEO audit done; fixes sent to Senthil on 8 July</t>
+          <t>Damco writes all answers — drafts shared with Will before posting</t>
         </is>
       </c>
-      <c r="C4" s="40" t="inlineStr">
+      <c r="C4" s="49" t="inlineStr">
         <is>
-          <t>Will to send corrected blog content</t>
+          <t>Review and approve draft answers — quick read and approve</t>
         </is>
       </c>
-      <c r="D4" s="40" t="inlineStr">
+      <c r="D4" s="49" t="inlineStr">
         <is>
-          <t>ASAP</t>
+          <t>Ongoing — weekly</t>
         </is>
       </c>
-      <c r="E4" s="43" t="inlineStr">
+      <c r="E4" s="49" t="inlineStr">
         <is>
-          <t>Waiting on Will</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F4" s="13" t="n"/>
@@ -860,28 +952,28 @@
       <c r="Y4" s="13" t="n"/>
       <c r="Z4" s="13" t="n"/>
     </row>
-    <row r="5" ht="14.25" customHeight="1" s="28">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="5" ht="50" customHeight="1" s="28">
+      <c r="A5" s="48" t="inlineStr">
         <is>
-          <t>FAQs</t>
+          <t>Reddit</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
         <is>
-          <t>Written and ready — schema code prepared for Senthil</t>
+          <t>Damco writes all answers — 3 questions shared with Will for topic approval</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C5" s="49" t="inlineStr">
         <is>
-          <t>Will to complete review and approve</t>
+          <t>Confirm the 3 questions are relevant — yes or no on each</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="49" t="inlineStr">
         <is>
-          <t>ASAP</t>
+          <t>29 July 2026</t>
         </is>
       </c>
-      <c r="E5" s="43" t="inlineStr">
+      <c r="E5" s="49" t="inlineStr">
         <is>
           <t>Waiting on Will</t>
         </is>
@@ -908,31 +1000,30 @@
       <c r="Y5" s="13" t="n"/>
       <c r="Z5" s="13" t="n"/>
     </row>
-    <row r="6" ht="14.25" customHeight="1" s="28">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="50" customHeight="1" s="28">
+      <c r="A6" s="48" t="inlineStr">
         <is>
-          <t>Website Fixes
-(Forms, CAPTCHA, Thank You pages, GTM)</t>
+          <t>Medium / Third-Party Articles</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="49" t="inlineStr">
         <is>
-          <t>Specifications sent to Senthil — GTM and Thank You page implementation included</t>
+          <t>Damco writes all articles — Medium account live, first draft being prepared</t>
         </is>
       </c>
-      <c r="C6" s="40" t="inlineStr">
+      <c r="C6" s="49" t="inlineStr">
         <is>
-          <t>Senthil to implement and confirm live date</t>
+          <t>Review each article draft before we publish — approve or request changes</t>
         </is>
       </c>
-      <c r="D6" s="40" t="inlineStr">
+      <c r="D6" s="49" t="inlineStr">
         <is>
-          <t>29 July 2026</t>
+          <t>Ongoing</t>
         </is>
       </c>
-      <c r="E6" s="41" t="inlineStr">
+      <c r="E6" s="49" t="inlineStr">
         <is>
-          <t>Waiting on Senthil</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F6" s="13" t="n"/>
@@ -957,28 +1048,28 @@
       <c r="Y6" s="13" t="n"/>
       <c r="Z6" s="13" t="n"/>
     </row>
-    <row r="7" ht="14.25" customHeight="1" s="28">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="7" ht="50" customHeight="1" s="28">
+      <c r="A7" s="48" t="inlineStr">
         <is>
-          <t>Quora</t>
+          <t>SEO Audit — Blog Pages</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="49" t="inlineStr">
         <is>
-          <t>Damco writes all answers — drafts shared with Will before posting</t>
+          <t>Audits done — fixes ranked by priority (Critical / Important / Good to have) and sent to Senthil</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="49" t="inlineStr">
         <is>
-          <t>Review and approve draft answers — quick read and approve</t>
+          <t>No action needed from Will — Senthil implements fixes</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="49" t="inlineStr">
         <is>
-          <t>Ongoing — weekly</t>
+          <t>Ongoing</t>
         </is>
       </c>
-      <c r="E7" s="41" t="inlineStr">
+      <c r="E7" s="49" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -1005,30 +1096,30 @@
       <c r="Y7" s="13" t="n"/>
       <c r="Z7" s="13" t="n"/>
     </row>
-    <row r="8" ht="14.25" customHeight="1" s="28">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="8" ht="50" customHeight="1" s="28">
+      <c r="A8" s="48" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>Monthly SEO Dashboard</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="49" t="inlineStr">
         <is>
-          <t>Damco writes all answers — 3 questions shared with Will for topic approval</t>
+          <t>Damco prepares and shares monthly — due 20th of each month</t>
         </is>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
-          <t>Confirm the 3 questions are relevant — yes or no on each</t>
+          <t>Review the report — flag any questions</t>
         </is>
       </c>
-      <c r="D8" s="40" t="inlineStr">
+      <c r="D8" s="49" t="inlineStr">
         <is>
-          <t>29 July 2026</t>
+          <t>20 August 2026</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
+      <c r="E8" s="49" t="inlineStr">
         <is>
-          <t>Waiting on Will</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F8" s="13" t="n"/>
@@ -1053,28 +1144,29 @@
       <c r="Y8" s="13" t="n"/>
       <c r="Z8" s="13" t="n"/>
     </row>
-    <row r="9" ht="14.25" customHeight="1" s="28">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="9" ht="50" customHeight="1" s="28">
+      <c r="A9" s="48" t="inlineStr">
         <is>
-          <t>Medium / Third-Party Articles</t>
+          <t>LLM Visibility
+(ChatGPT, Perplexity, Google AI)</t>
         </is>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>Damco writes all articles — Medium account live, first draft being prepared</t>
+          <t>Damco monitors Imago visibility in ChatGPT, Perplexity, and Google AI Overviews</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
-          <t>Review each article draft before we publish — approve or request changes</t>
+          <t>No action needed from Will's side</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="49" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>31 July 2026</t>
         </is>
       </c>
-      <c r="E9" s="41" t="inlineStr">
+      <c r="E9" s="49" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -1102,31 +1194,15 @@
       <c r="Z9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="28">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="50" t="inlineStr">
         <is>
-          <t>SEO Audit — Blog Pages</t>
+          <t>WAITING — Pending Will's input</t>
         </is>
       </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>Audits done — fixes ranked by priority (Critical / Important / Good to have) and sent to Senthil</t>
-        </is>
-      </c>
-      <c r="C10" s="40" t="inlineStr">
-        <is>
-          <t>No action needed from Will — Senthil implements fixes</t>
-        </is>
-      </c>
-      <c r="D10" s="40" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="E10" s="41" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+      <c r="B10" s="46" t="n"/>
+      <c r="C10" s="46" t="n"/>
+      <c r="D10" s="46" t="n"/>
+      <c r="E10" s="47" t="n"/>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
       <c r="H10" s="13" t="n"/>
@@ -1149,30 +1225,31 @@
       <c r="Y10" s="13" t="n"/>
       <c r="Z10" s="13" t="n"/>
     </row>
-    <row r="11" ht="14.25" customHeight="1" s="28">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="11" ht="50" customHeight="1" s="28">
+      <c r="A11" s="51" t="inlineStr">
         <is>
-          <t>Monthly SEO Dashboard</t>
+          <t>Blog — July post 1
+"Why Professional School Photography Matters"</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="52" t="inlineStr">
         <is>
-          <t>Damco prepares and shares monthly — due 20th of each month</t>
+          <t>Written and ready to publish — Will has shared blog content for review</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr">
+      <c r="C11" s="52" t="inlineStr">
         <is>
-          <t>Review the report — flag any questions</t>
+          <t>Senthil to upload to website once reviewed</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
+      <c r="D11" s="52" t="inlineStr">
         <is>
-          <t>20 August 2026</t>
+          <t>25 July 2026</t>
         </is>
       </c>
-      <c r="E11" s="41" t="inlineStr">
+      <c r="E11" s="52" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Senthil</t>
         </is>
       </c>
       <c r="F11" s="13" t="n"/>
@@ -1197,31 +1274,30 @@
       <c r="Y11" s="13" t="n"/>
       <c r="Z11" s="13" t="n"/>
     </row>
-    <row r="12" ht="14.25" customHeight="1" s="28">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="12" ht="50" customHeight="1" s="28">
+      <c r="A12" s="51" t="inlineStr">
         <is>
-          <t>LLM Visibility
-(ChatGPT, Perplexity, Google AI)</t>
+          <t>Blog — "How to Choose a School Photography Company in the UK"</t>
         </is>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B12" s="52" t="inlineStr">
         <is>
-          <t>Damco monitors Imago visibility in ChatGPT, Perplexity, and Google AI Overviews</t>
+          <t>Published on website — SEO audit done; fixes sent to Senthil on 8 July</t>
         </is>
       </c>
-      <c r="C12" s="40" t="inlineStr">
+      <c r="C12" s="52" t="inlineStr">
         <is>
-          <t>No action needed from Will's side</t>
+          <t>Will to send corrected blog content</t>
         </is>
       </c>
-      <c r="D12" s="40" t="inlineStr">
+      <c r="D12" s="52" t="inlineStr">
         <is>
-          <t>31 July 2026</t>
+          <t>ASAP</t>
         </is>
       </c>
-      <c r="E12" s="41" t="inlineStr">
+      <c r="E12" s="52" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Will</t>
         </is>
       </c>
       <c r="F12" s="13" t="n"/>
@@ -1246,12 +1322,32 @@
       <c r="Y12" s="13" t="n"/>
       <c r="Z12" s="13" t="n"/>
     </row>
-    <row r="13" ht="14.25" customHeight="1" s="28">
-      <c r="A13" s="13" t="n"/>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="13" t="n"/>
+    <row r="13" ht="50" customHeight="1" s="28">
+      <c r="A13" s="53" t="inlineStr">
+        <is>
+          <t>FAQs</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="inlineStr">
+        <is>
+          <t>Written and ready — schema code prepared for Senthil</t>
+        </is>
+      </c>
+      <c r="C13" s="53" t="inlineStr">
+        <is>
+          <t>Will to complete review and approve</t>
+        </is>
+      </c>
+      <c r="D13" s="53" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
+        <is>
+          <t>Waiting on Will</t>
+        </is>
+      </c>
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n"/>
       <c r="H13" s="13" t="n"/>
@@ -1275,11 +1371,15 @@
       <c r="Z13" s="13" t="n"/>
     </row>
     <row r="14" ht="14.25" customHeight="1" s="28">
-      <c r="A14" s="13" t="n"/>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="13" t="n"/>
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>PARKED — Website / on-page work (low period only)</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="n"/>
+      <c r="C14" s="46" t="n"/>
+      <c r="D14" s="46" t="n"/>
+      <c r="E14" s="47" t="n"/>
       <c r="F14" s="13" t="n"/>
       <c r="G14" s="13" t="n"/>
       <c r="H14" s="13" t="n"/>
@@ -1302,12 +1402,34 @@
       <c r="Y14" s="13" t="n"/>
       <c r="Z14" s="13" t="n"/>
     </row>
-    <row r="15" ht="14.25" customHeight="1" s="28">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="13" t="n"/>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="13" t="n"/>
+    <row r="15" ht="50" customHeight="1" s="28">
+      <c r="A15" s="55" t="inlineStr">
+        <is>
+          <t>Website Fixes
+(Forms, CAPTCHA, Thank You pages, GTM)
+⚑ Parked — to be done last week of August</t>
+        </is>
+      </c>
+      <c r="B15" s="55" t="inlineStr">
+        <is>
+          <t>Specifications sent to Senthil — GTM and Thank You page implementation included</t>
+        </is>
+      </c>
+      <c r="C15" s="55" t="inlineStr">
+        <is>
+          <t>Senthil to implement and confirm live date</t>
+        </is>
+      </c>
+      <c r="D15" s="55" t="inlineStr">
+        <is>
+          <t>Last week of August 2026</t>
+        </is>
+      </c>
+      <c r="E15" s="55" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
       <c r="F15" s="13" t="n"/>
       <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n"/>
@@ -28911,6 +29033,11 @@
       <c r="Z1000" s="13" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A14:E14"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In Progress,Waiting on Will,Waiting on Senthil,Done,Live,Planned,Damco Team,Imago team"</formula1>

</xml_diff>

<commit_message>
Slim down one-pager — short, concise descriptions throughout
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9QC9nTjspAMeTfXSbxYaC
</commit_message>
<xml_diff>
--- a/research/seo-activity-one-pager.xlsx
+++ b/research/seo-activity-one-pager.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,7 +28,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -50,7 +53,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
+        <fgColor rgb="00F5F6FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,11 +88,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,14 +462,14 @@
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Activity</t>
@@ -493,26 +496,25 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="52" customHeight="1">
+    <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Blog — July post 2
-"Why School Photography Matters / What to Look for in a New Photographer"</t>
+          <t>Blog 2 — Why School Photography Matters</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Writing in progress — draft to be shared with Will for approval</t>
+          <t>Writing draft</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Review and approve draft when shared</t>
+          <t>Approve draft when shared</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>25 July 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -521,26 +523,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="38" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Blog — July post 1
-"Why Professional School Photography Matters"</t>
+          <t>Blog 1 — Why Professional School Photography Matters</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Written and ready to publish — Will has shared blog content for review</t>
+          <t>Written — content received from Will</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Senthil to upload to website once reviewed</t>
+          <t>Senthil to upload</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>25 July 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -549,20 +550,20 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Blog — "How to Choose a School Photography Company in the UK"</t>
+          <t>Blog — How to Choose a School Photography Company</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Published on website — SEO audit done; fixes sent to Senthil on 8 July</t>
+          <t>Audit done, fixes sent to Senthil</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Will to send corrected blog content</t>
+          <t>Send corrected blog content</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -576,7 +577,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="38" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>FAQs</t>
@@ -584,12 +585,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Written and ready — schema code prepared for Senthil</t>
+          <t>Written, schema ready for Senthil</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Will to complete review and approve</t>
+          <t>Review and approve</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -603,7 +604,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Quora</t>
@@ -611,17 +612,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Damco writes all answers — drafts shared with Will before posting</t>
+          <t>Writing answers, sharing drafts before posting</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Review and approve draft answers — quick read and approve</t>
+          <t>Approve each draft</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Ongoing — weekly</t>
+          <t>Weekly</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -630,7 +631,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Reddit</t>
@@ -638,17 +639,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Damco writes all answers — 3 questions shared with Will for topic approval</t>
+          <t>3 questions shared for approval</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Confirm the 3 questions are relevant — yes or no on each</t>
+          <t>Approve or reject each question</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>29 July 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -657,7 +658,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="52" customHeight="1">
+    <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Medium / Third-Party Articles</t>
@@ -665,12 +666,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Damco writes all articles — Medium account live, first draft being prepared</t>
+          <t>Writing articles, Medium account live</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Review each article draft before we publish — approve or request changes</t>
+          <t>Approve each article before publish</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -684,7 +685,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="52" customHeight="1">
+    <row r="9" ht="38" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>SEO Audit — Blog Pages</t>
@@ -692,12 +693,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Audits done — fixes ranked by priority (Critical / Important / Good to have) and sent to Senthil</t>
+          <t>Fixes ranked Critical / Important / Good to have</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>No action needed from Will — Senthil implements fixes</t>
+          <t>No action needed — Senthil implements</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -711,7 +712,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="52" customHeight="1">
+    <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Monthly SEO Dashboard</t>
@@ -719,17 +720,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Damco prepares and shares monthly — due 20th of each month</t>
+          <t>Prepared and shared by 20th each month</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Review the report — flag any questions</t>
+          <t>Review and flag questions</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>20 August 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -738,26 +739,25 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="38" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>LLM Visibility
-(ChatGPT, Perplexity, Google AI)</t>
+          <t>LLM Visibility (ChatGPT, Perplexity, Google AI)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Damco monitors Imago visibility in ChatGPT, Perplexity, and Google AI Overviews</t>
+          <t>Monthly monitoring</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>No action needed from Will's side</t>
+          <t>No action needed</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>31 July 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -766,26 +766,25 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1">
+    <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Website Fixes
-(Forms, CAPTCHA, Thank You pages, GTM)</t>
+          <t>Website Fixes (Forms, CAPTCHA, Thank You, GTM)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Specifications sent to Senthil — GTM and Thank You page implementation included</t>
+          <t>Specs sent to Senthil</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Senthil to implement and confirm live date</t>
+          <t>Senthil to implement</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>August 2026</t>
+          <t>Aug 2026</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">

</xml_diff>